<commit_message>
Nuevo formato del reporte diario (diseño A4, azul marino)
- Acumulado del mes destacado arriba, con variación y avance vs año anterior.
- KPIs de ayer: venta, tickets y ticket promedio (con ticket promedio del mes vs año anterior).
- Variación del mes por sucursal, ordenada de mejor a peor (barras en HTML).
- Detalle con 4 columnas; el acumulado del año anterior va debajo del actual.
- Ancho fluido (máx. 600px): se lee bien en celular y en compu.
- Sin imágenes PNG salvo el logo (se ven aunque el correo bloquee imágenes).
- generar_acum2025.py ahora también suma los tickets del año anterior (col F).
- Si al historial le falta un día del mes, el mail sale igual pero sin tickets del mes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CfMPxk4Hk9SG3ihT4f3dvg
</commit_message>
<xml_diff>
--- a/Acumulado_interanual.xlsx
+++ b/Acumulado_interanual.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sales Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -474,7 +474,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="4">
@@ -496,7 +496,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>665</v>
       </c>
     </row>
     <row r="5">
@@ -518,7 +518,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="6">
@@ -540,7 +540,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>919</v>
       </c>
     </row>
     <row r="7">
@@ -562,7 +562,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>565</v>
       </c>
     </row>
     <row r="8">
@@ -584,7 +584,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9">
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>5365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>